<commit_message>
feat(matrix): Holding Brake axis, magnetic-absolute sensor row, Brushed (DC) row resolved
docs/tools/add_holding_brake_axis.py (idempotent, openpyxl, timestamped
backup) adds the Holding Brake sheet with a Fail-state column, resolves
the Motor sheet's Brushed (DC) gate-driver cell (TBD since 2026-08-16,
TODO 12.6.a) to the TI DRV8874-Q1 integrated bridge [63] with shunt qty 0
(IPROPI mirror), appends a Magnetic absolute (SPI/SSI) row for the
AEAT-8800-Q24 [64], records on the Amperage sheet that the Motor sheet's
bridge row overrides its brushless-shaped power-stage columns for brushed
builds, and lists the new axis in the Legend. JSON re-exported
(decision_matrix_to_json.py --check passes); root README Build Options
updated.

Plan: Serenity-UAV docs/plans/2026-09-17-001-…-plan.md U2 (KTD3, KTD7).

AI note: authored by Claude Opus 5 (claude-opus-5) under the direction of
Steve Griffing, PE(CSE), CISSP-ISSEP, CPP.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/decision-matrix.xlsx
+++ b/docs/decision-matrix.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Legend" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Voltage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Amperage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Motor" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Shaft Sensor" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Protocol" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Control" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="EMI Hardening" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Wire Egress" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Form Factor" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voltage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amperage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motor" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shaft Sensor" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Holding Brake" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EMI Hardening" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wire Egress" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form Factor" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -31,7 +32,7 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -166,6 +167,10 @@
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -244,7 +249,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -434,6 +439,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -709,7 +718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24" customWidth="1" style="30" min="1" max="1"/>
@@ -730,6 +739,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="48" customHeight="1" s="31">
       <c r="A4" s="34" t="inlineStr">
         <is>
@@ -742,6 +752,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="15" customHeight="1" s="31">
       <c r="A6" s="34" t="inlineStr">
         <is>
@@ -797,6 +808,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="31">
       <c r="A12" s="34" t="inlineStr">
         <is>
@@ -811,6 +823,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="31">
       <c r="A15" s="34" t="inlineStr">
         <is>
@@ -902,10 +915,31 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="15" customHeight="1" s="31">
       <c r="A24" s="44" t="inlineStr">
         <is>
           <t>Amended 2026-08-16: added the Motor and Shaft Sensor axis sheets. Cells reading 'TBD -- requires primary-source verification' are genuinely unsourced, not placeholders to be filled in from memory (AGENTS.md Sec.1.3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="61" t="inlineStr">
+        <is>
+          <t>Holding Brake</t>
+        </is>
+      </c>
+      <c r="B25" s="63" t="inlineStr">
+        <is>
+          <t>None / low-side solenoid driver: actuation, fail-state (the safety property), MCU pins, driver part, connector, firmware sequencing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26"/>
+    <row r="27">
+      <c r="A27" s="65" t="inlineStr">
+        <is>
+          <t>Amended 2026-09-17: added the Holding Brake axis; resolved the Motor sheet's Brushed (DC) row (DRV8874-Q1 [63]); added the magnetic-absolute shaft-sensor row (AEAT-8800-Q24 [64]).</t>
         </is>
       </c>
     </row>
@@ -932,6 +966,177 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" style="31" min="1" max="1"/>
+    <col width="30" customWidth="1" style="31" min="2" max="2"/>
+    <col width="34" customWidth="1" style="31" min="3" max="3"/>
+    <col width="38" customWidth="1" style="31" min="4" max="4"/>
+    <col width="30" customWidth="1" style="31" min="5" max="5"/>
+    <col width="44" customWidth="1" style="31" min="6" max="6"/>
+    <col width="18" customWidth="1" style="31" min="7" max="7"/>
+    <col width="22" customWidth="1" style="31" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="60" t="inlineStr">
+        <is>
+          <t>Wire Egress Decision Matrix</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>Build axis: Wire Egress (Opposite-end / Same-end, opposite faces)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="62" t="inlineStr">
+        <is>
+          <t>Egress Pattern</t>
+        </is>
+      </c>
+      <c r="B4" s="62" t="inlineStr">
+        <is>
+          <t>Terminal Face Assignment</t>
+        </is>
+      </c>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>Board Re-partition Required</t>
+        </is>
+      </c>
+      <c r="D4" s="62" t="inlineStr">
+        <is>
+          <t>Inner-Plane Shield Requirement</t>
+        </is>
+      </c>
+      <c r="E4" s="62" t="inlineStr">
+        <is>
+          <t>Additional BOM Component</t>
+        </is>
+      </c>
+      <c r="F4" s="62" t="inlineStr">
+        <is>
+          <t>Workflow Steps</t>
+        </is>
+      </c>
+      <c r="G4" s="62" t="inlineStr">
+        <is>
+          <t>REFERENCES.md Tags</t>
+        </is>
+      </c>
+      <c r="H4" s="62" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="63" t="inlineStr">
+        <is>
+          <t>Opposite-end (default)</t>
+        </is>
+      </c>
+      <c r="B5" s="63" t="inlineStr">
+        <is>
+          <t>Pack J5A/J5B on F.Cu at one board end; phases J4A/J4B/J4C on F.Cu at the other. Both groups sit directly on their own pours.</t>
+        </is>
+      </c>
+      <c r="C5" s="63" t="inlineStr">
+        <is>
+          <t>None. This is the as-built arrangement on builds/6s/50A/CAN_485_faraday/.</t>
+        </is>
+      </c>
+      <c r="D5" s="63" t="inlineStr">
+        <is>
+          <t>None arising from egress. The In1.Cu GND plane and the In2.Cu GND pour above y 60.5 mm serve their normal return and shielding roles; no terminal group is stacked over another.</t>
+        </is>
+      </c>
+      <c r="E5" s="63" t="inlineStr">
+        <is>
+          <t>None beyond the selected EMI Hardening tier</t>
+        </is>
+      </c>
+      <c r="F5" s="63" t="inlineStr">
+        <is>
+          <t>No egress-specific step. Terminal placement follows the power-stage placement; verify each terminal lands on its own pour per docs/tools/conductor_sizing.py.</t>
+        </is>
+      </c>
+      <c r="G5" s="63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" s="63" t="inlineStr">
+        <is>
+          <t>Candidate (unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="63" t="inlineStr">
+        <is>
+          <t>Same-end, opposite faces</t>
+        </is>
+      </c>
+      <c r="B6" s="63" t="inlineStr">
+        <is>
+          <t>Both groups leave the same board end. Phases J4A/J4B/J4C stay on F.Cu on their existing pours (unchanged); pack J5A/J5B move to B.Cu directly opposite. The two inner GND planes lie between them.</t>
+        </is>
+      </c>
+      <c r="C6" s="63" t="inlineStr">
+        <is>
+          <t>Yes. B.Cu at the terminal end currently holds the MCU U1, the secure element U2 and the probe pads J1; all three must vacate to the logic end. VM distribution must also be extended to reach a B.Cu pad at that end -- today the VM pour stops at y 60.3 mm (F.Cu) / 60.5 mm (In2.Cu).</t>
+        </is>
+      </c>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>MANDATORY and NOT currently met. The unnamed rule area at x 20.75-51.15, y 76.50-86.55 mm sets `copperpour not_allowed` on ALL FOUR copper layers, so In1.Cu and In2.Cu are cut away exactly where the two terminal groups would face each other. That rule area must be restricted to the outer layers, the inner GND planes must pour solid through the terminal window, and phase via transitions must be kept out of that window so no antipad perforates the shield.</t>
+        </is>
+      </c>
+      <c r="E6" s="63" t="inlineStr">
+        <is>
+          <t>Common-mode choke on the pack input -- TBD -- requires primary-source verification (AGENTS.md Sec.1.3). No choke has been sourced or verified in this repo.</t>
+        </is>
+      </c>
+      <c r="F6" s="63" t="inlineStr">
+        <is>
+          <t>Define a stackup FIRST -- the board currently has none (4 copper layers declared, `(thickness 1.6)` is KiCad's default, no dielectric height or copper weight specified). Then: fix the rule area's layer scope; re-place U1/U2/J1; extend VM to B.Cu; stitch In1/In2 with a GND via fence around the terminal window; re-run conductor_sizing.py and isolation_envelope.py; negative-control every new DRC rule before trusting it.</t>
+        </is>
+      </c>
+      <c r="G6" s="63" t="inlineStr">
+        <is>
+          <t>[9], [49]</t>
+        </is>
+      </c>
+      <c r="H6" s="63" t="inlineStr">
+        <is>
+          <t>Open / unresolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="64" t="inlineStr">
+        <is>
+          <t>Note: Rejected third arrangement: same end, both groups on the outer faces but split onto the two long edges. Five terminals in one row need 2 x 7.0 mm + 3 x 5.0 mm = 29.0 mm of pad on a 32.00 mm edge, leaving 0.50 mm per gap once four inter-pad gaps and two edge margins are taken -- not dressable with 6 sq.mm (~10 AWG) conductor, its solder fillet and its strain relief. Widening the board to suit is governed by docs/solutions/architecture-patterns/isolation-geometry-sets-board-aspect.md, which prices width at 3.0x the length it saves. See docs/design-single-end-wire-egress-variant.md Sec.7.2. -- Board thickness is NOT a usable lever for face-to-face separation: with a grounded plane between the faces the direct coupling path is already terminated, whereas doubling the laminate thickness only halves a parallel-plate capacitance. Restore the plane rather than thicken the board.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1761,7 +1966,7 @@
       </c>
       <c r="L5" s="50" t="inlineStr">
         <is>
-          <t>[20], [21], [22], [23]</t>
+          <t>[20], [21], [22], [23], [62], [63]</t>
         </is>
       </c>
       <c r="M5" s="37" t="inlineStr">
@@ -2106,10 +2311,11 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="60" customHeight="1" s="31">
-      <c r="A13" s="57" t="inlineStr">
-        <is>
-          <t>Shunt part: Vishay WSLP2512 [23] (3.0W package rating). "Shunt Qty Needed" = ROUNDUP(Shunt Power / 3W, 0); at 80A/120A this correctly computes 2x and 3x devices in parallel (7.2W / 3 tiers exceeds a single package's rating). FET parallel count and gate-driver reuse are a BOM-commonality choice (AGENTS.md §4 judgment call), not a datasheet requirement -- a smaller SO-8 FET would be leaner for the 10A-30A tiers if part-count commonality were not prioritized.</t>
+      <c r="A13" s="66" t="inlineStr">
+        <is>
+          <t>Shunt part: Vishay WSLP2512 [23] (3.0W package rating). "Shunt Qty Needed" = ROUNDUP(Shunt Power / 3W, 0); at 80A/120A this correctly computes 2x and 3x devices in parallel (7.2W / 3 tiers exceeds a single package's rating). FET parallel count and gate-driver reuse are a BOM-commonality choice (AGENTS.md §4 judgment call), not a datasheet requirement -- a smaller SO-8 FET would be leaner for the 10A-30A tiers if part-count commonality were not prioritized. -- BRUSHED BUILDS (2026-09-17): the FET Part, Gate Driver Part, Shunt and Current-Sense Amp columns of this sheet are brushless-shaped and are OVERRIDDEN by the Motor sheet's bridge row for a Brushed (DC) build (Tier 1: DRV8874-Q1 [63] integrated bridge, no shunt). This sheet still governs the copper and connector class for the tier.</t>
         </is>
       </c>
     </row>
@@ -2269,9 +2475,9 @@
           <t>4 (2 high + 2 low)</t>
         </is>
       </c>
-      <c r="D6" s="43" t="inlineStr">
-        <is>
-          <t>TBD -- requires primary-source verification (AGENTS.md Sec.1.3). No H-bridge gate driver has been sourced or verified in this repo. NOTE, not yet vetted: a 3-phase driver such as the DRV8353S [21] can drive an H-bridge by using two of its three half-bridges and leaving the third unused -- this reuses an already-verified part at the cost of wasted silicon and board area, and must be checked against [21] before adoption.</t>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>TI DRV8874-Q1 [63] integrated N-channel H-bridge (non-Q1 twin DRV8874 [62]): 4.5-37 V VM, 6 A peak, 100 mOhm typ per FET, PH/EN or PWM control, IPROPI current mirror 450 uA/A, VREF/ITRIP current regulation, UVLO/CPUV/OCP/TSD. Tier 1 (2S-6S, 10-20 A) per docs/OpenSecureESC-Brushed-Specifications.md Sec.1; every fault coasts the bridge ([63] Table 7).</t>
         </is>
       </c>
       <c r="E6" s="43" t="inlineStr">
@@ -2279,9 +2485,9 @@
           <t>2 (M+ / M-)</t>
         </is>
       </c>
-      <c r="F6" s="43" t="inlineStr">
-        <is>
-          <t>1-2 (bridge-leg or in-line)</t>
+      <c r="F6" s="63" t="inlineStr">
+        <is>
+          <t>0 -- the driver's IPROPI current mirror replaces the shunt and current-sense amplifier of the brushless tiers ([63] Sec.7.3.3.1)</t>
         </is>
       </c>
       <c r="G6" s="43" t="inlineStr">
@@ -2289,14 +2495,14 @@
           <t>None -- direction and magnitude set by bridge polarity and duty cycle; no rotor position needed for basic operation</t>
         </is>
       </c>
-      <c r="H6" s="43" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I6" s="43" t="inlineStr">
-        <is>
-          <t>Open / unresolved</t>
+      <c r="H6" s="63" t="inlineStr">
+        <is>
+          <t>[62], [63]</t>
+        </is>
+      </c>
+      <c r="I6" s="63" t="inlineStr">
+        <is>
+          <t>Verified (local PDF)</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="30" min="1" max="1"/>
@@ -2550,6 +2756,48 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="63" t="inlineStr">
+        <is>
+          <t>Magnetic absolute (SPI/SSI)</t>
+        </is>
+      </c>
+      <c r="B9" s="63" t="inlineStr">
+        <is>
+          <t>Single-turn absolute angle from an on-axis Hall sensor IC reading a diametric two-pole magnet on the shaft end; 10- to 16-bit absolute word over SSI/SPI, optional ABI/UVW/PWM outputs. Multi-turn position is accumulated in firmware.</t>
+        </is>
+      </c>
+      <c r="C9" s="63" t="inlineStr">
+        <is>
+          <t>3 (SCLK, DO, NSL/CS) for SSI, 4 with DI for SPI; sensor supply 3.3 V. The sensor may sit off-board on a short cable.</t>
+        </is>
+      </c>
+      <c r="D9" s="63" t="inlineStr">
+        <is>
+          <t>Broadcom AEAT-8800-Q24 [64], QFN-24 5 x 5 mm, 3.3 V or 5 V operation, SSI 3-wire absolute output. Series resistors and ESD protection on each line per docs/design-speed-sensor-integration.md.</t>
+        </is>
+      </c>
+      <c r="E9" s="63" t="inlineStr">
+        <is>
+          <t>6-pin keyed (3V3, GND, SCLK, DO, NSL, DI) with shield/drain optional</t>
+        </is>
+      </c>
+      <c r="F9" s="63" t="inlineStr">
+        <is>
+          <t>Read the absolute word each control tick; unwrap turns across the 0/full-scale boundary; home the multi-turn count from an outer absolute reference (a host sensor over the bus) at power-up; declare 'stationary' from this sensor, not from motor current.</t>
+        </is>
+      </c>
+      <c r="G9" s="63" t="inlineStr">
+        <is>
+          <t>[64]</t>
+        </is>
+      </c>
+      <c r="H9" s="63" t="inlineStr">
+        <is>
+          <t>Verified (local PDF)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2558,6 +2806,193 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" style="31" min="1" max="1"/>
+    <col width="34" customWidth="1" style="31" min="2" max="2"/>
+    <col width="40" customWidth="1" style="31" min="3" max="3"/>
+    <col width="26" customWidth="1" style="31" min="4" max="4"/>
+    <col width="40" customWidth="1" style="31" min="5" max="5"/>
+    <col width="30" customWidth="1" style="31" min="6" max="6"/>
+    <col width="44" customWidth="1" style="31" min="7" max="7"/>
+    <col width="18" customWidth="1" style="31" min="8" max="8"/>
+    <col width="22" customWidth="1" style="31" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="60" t="inlineStr">
+        <is>
+          <t>Holding Brake Decision Matrix</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>Build axis: Holding Brake (None / Low-side solenoid driver, spring-applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="62" t="inlineStr">
+        <is>
+          <t>Brake Option</t>
+        </is>
+      </c>
+      <c r="B4" s="62" t="inlineStr">
+        <is>
+          <t>Actuation</t>
+        </is>
+      </c>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>Fail-state</t>
+        </is>
+      </c>
+      <c r="D4" s="62" t="inlineStr">
+        <is>
+          <t>MCU Pins Required</t>
+        </is>
+      </c>
+      <c r="E4" s="62" t="inlineStr">
+        <is>
+          <t>Additional BOM Component</t>
+        </is>
+      </c>
+      <c r="F4" s="62" t="inlineStr">
+        <is>
+          <t>Connector</t>
+        </is>
+      </c>
+      <c r="G4" s="62" t="inlineStr">
+        <is>
+          <t>Firmware Workflow Steps</t>
+        </is>
+      </c>
+      <c r="H4" s="62" t="inlineStr">
+        <is>
+          <t>REFERENCES.md Tags</t>
+        </is>
+      </c>
+      <c r="I4" s="62" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="63" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="B5" s="63" t="inlineStr">
+        <is>
+          <t>No holding brake. The load is held by the motor's own drag, a self-locking transmission, or nothing.</t>
+        </is>
+      </c>
+      <c r="C5" s="63" t="inlineStr">
+        <is>
+          <t>Not applicable -- the build has no brake to fail. A non-self-locking transmission on a load that must hold unpowered may NOT select this row.</t>
+        </is>
+      </c>
+      <c r="D5" s="63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E5" s="63" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F5" s="63" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G5" s="63" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H5" s="63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" s="63" t="inlineStr">
+        <is>
+          <t>No part needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="63" t="inlineStr">
+        <is>
+          <t>Low-side solenoid driver, spring-applied</t>
+        </is>
+      </c>
+      <c r="B6" s="63" t="inlineStr">
+        <is>
+          <t>Spring-applied, power-released pin brake. A pull solenoid retracts the pin while its coil is energised; the spring engages the pin when the coil is released. The coil is switched on its low side.</t>
+        </is>
+      </c>
+      <c r="C6" s="63" t="inlineStr">
+        <is>
+          <t>De-energised = engaged. The driver input carries a pull-down so an MCU reset, brown-out or floating GPIO engages the brake without firmware; the coil's inductive kick is clamped; brake state (drive-pin readback) is published on the bus. Engage-on-fault: the motor driver's nFAULT is a brake-engage input for firmware.</t>
+        </is>
+      </c>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>1 digital out (BRAKE_EN) plus 1 digital in or ADC for state readback; optionally 1 ADC for the coil supply rail so the pin is never dropped into a driven castellation.</t>
+        </is>
+      </c>
+      <c r="E6" s="63" t="inlineStr">
+        <is>
+          <t>TI TPL7407L [66]: 40 V 7-channel NMOS low-side array, 600 mA per channel (channels paralleled for the load), 1 MOhm input pull-down per channel, internal clamp diodes to COM. Return COM to the pack-side rail so the clamp sits above the coil supply and inside the COM range (8.5-40 V, [66] Sec.6.3). The solenoid itself is a host-side part outside this axis (Serenity-UAV item BRK-4); this row carries only the driver.</t>
+        </is>
+      </c>
+      <c r="F6" s="63" t="inlineStr">
+        <is>
+          <t>2-pin (COIL+, COIL-) keyed header; polarity marked</t>
+        </is>
+      </c>
+      <c r="G6" s="63" t="inlineStr">
+        <is>
+          <t>Release only on an authenticated release command after the loop has unloaded the pin; sequence release -&gt; move -&gt; settle (encoder stationary) -&gt; engage; engage on nFAULT, on bus loss after a timeout, and on coil-rail droop below the solenoid hold-in voltage; publish brake state every telemetry frame.</t>
+        </is>
+      </c>
+      <c r="H6" s="63" t="inlineStr">
+        <is>
+          <t>[66]</t>
+        </is>
+      </c>
+      <c r="I6" s="63" t="inlineStr">
+        <is>
+          <t>Verified (local PDF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="64" t="inlineStr">
+        <is>
+          <t>Note: A brake on the actuator shaft protects against loss of drive, not against a broken transmission downstream of it. The 'Fail-state' column is the safety property this axis exists to record -- a build that selects the solenoid row must reproduce every item in it, not just the part number. First instance: builds/6s/10A/BRUSHED_CAN_485_isolation/ (Serenity-UAV nacelle tilt).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2983,7 +3418,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3153,7 +3588,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3379,175 +3814,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" style="31" min="1" max="1"/>
-    <col width="30" customWidth="1" style="31" min="2" max="2"/>
-    <col width="34" customWidth="1" style="31" min="3" max="3"/>
-    <col width="38" customWidth="1" style="31" min="4" max="4"/>
-    <col width="30" customWidth="1" style="31" min="5" max="5"/>
-    <col width="44" customWidth="1" style="31" min="6" max="6"/>
-    <col width="18" customWidth="1" style="31" min="7" max="7"/>
-    <col width="22" customWidth="1" style="31" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="60" t="inlineStr">
-        <is>
-          <t>Wire Egress Decision Matrix</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="61" t="inlineStr">
-        <is>
-          <t>Build axis: Wire Egress (Opposite-end / Same-end, opposite faces)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="62" t="inlineStr">
-        <is>
-          <t>Egress Pattern</t>
-        </is>
-      </c>
-      <c r="B4" s="62" t="inlineStr">
-        <is>
-          <t>Terminal Face Assignment</t>
-        </is>
-      </c>
-      <c r="C4" s="62" t="inlineStr">
-        <is>
-          <t>Board Re-partition Required</t>
-        </is>
-      </c>
-      <c r="D4" s="62" t="inlineStr">
-        <is>
-          <t>Inner-Plane Shield Requirement</t>
-        </is>
-      </c>
-      <c r="E4" s="62" t="inlineStr">
-        <is>
-          <t>Additional BOM Component</t>
-        </is>
-      </c>
-      <c r="F4" s="62" t="inlineStr">
-        <is>
-          <t>Workflow Steps</t>
-        </is>
-      </c>
-      <c r="G4" s="62" t="inlineStr">
-        <is>
-          <t>REFERENCES.md Tags</t>
-        </is>
-      </c>
-      <c r="H4" s="62" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="63" t="inlineStr">
-        <is>
-          <t>Opposite-end (default)</t>
-        </is>
-      </c>
-      <c r="B5" s="63" t="inlineStr">
-        <is>
-          <t>Pack J5A/J5B on F.Cu at one board end; phases J4A/J4B/J4C on F.Cu at the other. Both groups sit directly on their own pours.</t>
-        </is>
-      </c>
-      <c r="C5" s="63" t="inlineStr">
-        <is>
-          <t>None. This is the as-built arrangement on builds/6s/50A/CAN_485_faraday/.</t>
-        </is>
-      </c>
-      <c r="D5" s="63" t="inlineStr">
-        <is>
-          <t>None arising from egress. The In1.Cu GND plane and the In2.Cu GND pour above y 60.5 mm serve their normal return and shielding roles; no terminal group is stacked over another.</t>
-        </is>
-      </c>
-      <c r="E5" s="63" t="inlineStr">
-        <is>
-          <t>None beyond the selected EMI Hardening tier</t>
-        </is>
-      </c>
-      <c r="F5" s="63" t="inlineStr">
-        <is>
-          <t>No egress-specific step. Terminal placement follows the power-stage placement; verify each terminal lands on its own pour per docs/tools/conductor_sizing.py.</t>
-        </is>
-      </c>
-      <c r="G5" s="63" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H5" s="63" t="inlineStr">
-        <is>
-          <t>Candidate (unverified)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="63" t="inlineStr">
-        <is>
-          <t>Same-end, opposite faces</t>
-        </is>
-      </c>
-      <c r="B6" s="63" t="inlineStr">
-        <is>
-          <t>Both groups leave the same board end. Phases J4A/J4B/J4C stay on F.Cu on their existing pours (unchanged); pack J5A/J5B move to B.Cu directly opposite. The two inner GND planes lie between them.</t>
-        </is>
-      </c>
-      <c r="C6" s="63" t="inlineStr">
-        <is>
-          <t>Yes. B.Cu at the terminal end currently holds the MCU U1, the secure element U2 and the probe pads J1; all three must vacate to the logic end. VM distribution must also be extended to reach a B.Cu pad at that end -- today the VM pour stops at y 60.3 mm (F.Cu) / 60.5 mm (In2.Cu).</t>
-        </is>
-      </c>
-      <c r="D6" s="63" t="inlineStr">
-        <is>
-          <t>MANDATORY and NOT currently met. The unnamed rule area at x 20.75-51.15, y 76.50-86.55 mm sets `copperpour not_allowed` on ALL FOUR copper layers, so In1.Cu and In2.Cu are cut away exactly where the two terminal groups would face each other. That rule area must be restricted to the outer layers, the inner GND planes must pour solid through the terminal window, and phase via transitions must be kept out of that window so no antipad perforates the shield.</t>
-        </is>
-      </c>
-      <c r="E6" s="63" t="inlineStr">
-        <is>
-          <t>Common-mode choke on the pack input -- TBD -- requires primary-source verification (AGENTS.md Sec.1.3). No choke has been sourced or verified in this repo.</t>
-        </is>
-      </c>
-      <c r="F6" s="63" t="inlineStr">
-        <is>
-          <t>Define a stackup FIRST -- the board currently has none (4 copper layers declared, `(thickness 1.6)` is KiCad's default, no dielectric height or copper weight specified). Then: fix the rule area's layer scope; re-place U1/U2/J1; extend VM to B.Cu; stitch In1/In2 with a GND via fence around the terminal window; re-run conductor_sizing.py and isolation_envelope.py; negative-control every new DRC rule before trusting it.</t>
-        </is>
-      </c>
-      <c r="G6" s="63" t="inlineStr">
-        <is>
-          <t>[9], [49]</t>
-        </is>
-      </c>
-      <c r="H6" s="63" t="inlineStr">
-        <is>
-          <t>Open / unresolved</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="64" t="inlineStr">
-        <is>
-          <t>Note: Rejected third arrangement: same end, both groups on the outer faces but split onto the two long edges. Five terminals in one row need 2 x 7.0 mm + 3 x 5.0 mm = 29.0 mm of pad on a 32.00 mm edge, leaving 0.50 mm per gap once four inter-pad gaps and two edge margins are taken -- not dressable with 6 sq.mm (~10 AWG) conductor, its solder fillet and its strain relief. Widening the board to suit is governed by docs/solutions/architecture-patterns/isolation-geometry-sets-board-aspect.md, which prices width at 3.0x the length it saves. See docs/design-single-end-wire-egress-variant.md Sec.7.2. -- Board thickness is NOT a usable lever for face-to-face separation: with a grounded plane between the faces the direct coupling path is already terminated, whereas doubling the laminate thickness only halves a parallel-plate capacitance. Restore the plane rather than thicken the board.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>